<commit_message>
feat(calendar): add persian datepicker button and auto-slash formatting to company registration date
</commit_message>
<xml_diff>
--- a/Git_hespy.xlsx
+++ b/Git_hespy.xlsx
@@ -13,6 +13,8 @@
   </bookViews>
   <sheets>
     <sheet name="Git_hespy" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -24,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="15">
   <si>
     <t>کلمه کلیدی در کیت هاب</t>
   </si>
@@ -46,18 +48,121 @@
   <si>
     <t>اضافه بر مرحله قبل مشکل تم برنامه حل شد و تم بصورت ماندگار در برنامه اعمال می شود</t>
   </si>
+  <si>
+    <r>
+      <t>هر زمان که کلمه کلیدی </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9.9"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>hespy2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> را بفرمایید، برنامه دقیقاً به همین وضعیت و مرحله با دستور زیر بازگردانی و پول خواهد شد</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">این تست 
+متن چند خطی
+برای ورود به یک سلول اکسل هست
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">سلام
+این متن
+چند خطی </t>
+  </si>
+  <si>
+    <t>لطفا این مرحله برنامه رو با کلمه کلیدی و تگ زیر در گیتهاب پوش کن ، تا هر وقت به تو کلمه کلیدی رو گفتم ، برنامه رو تا این مرحله برام پول بکنی
+کلمه کلیدی 
+hespy2</t>
+  </si>
+  <si>
+    <t>git fetch --tags
+git checkout tags/hespy2</t>
+  </si>
+  <si>
+    <r>
+      <t>هر زمان که تمایل داشته باشید این مرحله دقیقاً بازگردانی شود، با گفتن کلمه کلیدی </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9.9"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>hespy1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t>، پروژه دقیقاً از روی تگ و کامیت </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9.9"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>hespy1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Segoe UI"/>
+        <family val="2"/>
+      </rPr>
+      <t> با دستور زیر برای شما پول و ریستور خواهد شد:</t>
+    </r>
+  </si>
+  <si>
+    <t>git fetch --tags
+git checkout tags/hespy1</t>
+  </si>
+  <si>
+    <t>دستور پول از گیتهاب</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9.9"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="9.9"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -80,7 +185,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -90,6 +195,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -371,14 +482,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D100"/>
+  <dimension ref="A1:E100"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="14.42578125" customWidth="1"/>
-    <col min="4" max="4" width="124.85546875" customWidth="1"/>
+    <col min="4" max="4" width="56.42578125" customWidth="1"/>
+    <col min="5" max="5" width="30.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -391,8 +503,11 @@
       <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
@@ -406,8 +521,11 @@
       <c r="D2" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E2" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
@@ -421,8 +539,11 @@
       <c r="D3" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E3" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
@@ -435,7 +556,7 @@
       </c>
       <c r="D4" s="1"/>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
@@ -448,7 +569,7 @@
       </c>
       <c r="D5" s="1"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
@@ -461,7 +582,7 @@
       </c>
       <c r="D6" s="1"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>4</v>
       </c>
@@ -474,7 +595,7 @@
       </c>
       <c r="D7" s="1"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>4</v>
       </c>
@@ -487,7 +608,7 @@
       </c>
       <c r="D8" s="1"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>4</v>
       </c>
@@ -500,7 +621,7 @@
       </c>
       <c r="D9" s="1"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>4</v>
       </c>
@@ -513,7 +634,7 @@
       </c>
       <c r="D10" s="1"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>4</v>
       </c>
@@ -526,7 +647,7 @@
       </c>
       <c r="D11" s="1"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>4</v>
       </c>
@@ -539,7 +660,7 @@
       </c>
       <c r="D12" s="1"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>4</v>
       </c>
@@ -552,7 +673,7 @@
       </c>
       <c r="D13" s="1"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>4</v>
       </c>
@@ -565,7 +686,7 @@
       </c>
       <c r="D14" s="1"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>4</v>
       </c>
@@ -578,7 +699,7 @@
       </c>
       <c r="D15" s="1"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>4</v>
       </c>
@@ -1687,4 +1808,487 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A3:C90"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="36.42578125" customWidth="1"/>
+    <col min="2" max="2" width="103.28515625" customWidth="1"/>
+    <col min="3" max="3" width="41.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="1:3" ht="66" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="82.5" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B6" s="4"/>
+      <c r="C6" s="4"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="4"/>
+      <c r="B8" s="4"/>
+      <c r="C8" s="4"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="4"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="4"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="4"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="4"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="4"/>
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="4"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="4"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="4"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="4"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="4"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="4"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="4"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="4"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="4"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="4"/>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="4"/>
+      <c r="B22" s="4"/>
+      <c r="C22" s="4"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="4"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="4"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="4"/>
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="4"/>
+      <c r="B26" s="4"/>
+      <c r="C26" s="4"/>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="4"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="4"/>
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="4"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="4"/>
+      <c r="B30" s="4"/>
+      <c r="C30" s="4"/>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="4"/>
+      <c r="B31" s="4"/>
+      <c r="C31" s="4"/>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="4"/>
+      <c r="B32" s="4"/>
+      <c r="C32" s="4"/>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="4"/>
+      <c r="B33" s="4"/>
+      <c r="C33" s="4"/>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="4"/>
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="4"/>
+      <c r="B35" s="4"/>
+      <c r="C35" s="4"/>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="4"/>
+      <c r="B36" s="4"/>
+      <c r="C36" s="4"/>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="4"/>
+      <c r="B37" s="4"/>
+      <c r="C37" s="4"/>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="4"/>
+      <c r="B38" s="4"/>
+      <c r="C38" s="4"/>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="4"/>
+      <c r="B39" s="4"/>
+      <c r="C39" s="4"/>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" s="4"/>
+      <c r="B40" s="4"/>
+      <c r="C40" s="4"/>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="4"/>
+      <c r="B41" s="4"/>
+      <c r="C41" s="4"/>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" s="4"/>
+      <c r="B42" s="4"/>
+      <c r="C42" s="4"/>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" s="4"/>
+      <c r="B43" s="4"/>
+      <c r="C43" s="4"/>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" s="4"/>
+      <c r="B44" s="4"/>
+      <c r="C44" s="4"/>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" s="4"/>
+      <c r="B45" s="4"/>
+      <c r="C45" s="4"/>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" s="4"/>
+      <c r="B46" s="4"/>
+      <c r="C46" s="4"/>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" s="4"/>
+      <c r="B47" s="4"/>
+      <c r="C47" s="4"/>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" s="4"/>
+      <c r="B48" s="4"/>
+      <c r="C48" s="4"/>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" s="4"/>
+      <c r="B49" s="4"/>
+      <c r="C49" s="4"/>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" s="4"/>
+      <c r="B50" s="4"/>
+      <c r="C50" s="4"/>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" s="4"/>
+      <c r="B51" s="4"/>
+      <c r="C51" s="4"/>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" s="4"/>
+      <c r="B52" s="4"/>
+      <c r="C52" s="4"/>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" s="4"/>
+      <c r="B53" s="4"/>
+      <c r="C53" s="4"/>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" s="4"/>
+      <c r="B54" s="4"/>
+      <c r="C54" s="4"/>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" s="4"/>
+      <c r="B55" s="4"/>
+      <c r="C55" s="4"/>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" s="4"/>
+      <c r="B56" s="4"/>
+      <c r="C56" s="4"/>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" s="4"/>
+      <c r="B57" s="4"/>
+      <c r="C57" s="4"/>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" s="4"/>
+      <c r="B58" s="4"/>
+      <c r="C58" s="4"/>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" s="4"/>
+      <c r="B59" s="4"/>
+      <c r="C59" s="4"/>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" s="4"/>
+      <c r="B60" s="4"/>
+      <c r="C60" s="4"/>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" s="4"/>
+      <c r="B61" s="4"/>
+      <c r="C61" s="4"/>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62" s="4"/>
+      <c r="B62" s="4"/>
+      <c r="C62" s="4"/>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63" s="4"/>
+      <c r="B63" s="4"/>
+      <c r="C63" s="4"/>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64" s="4"/>
+      <c r="B64" s="4"/>
+      <c r="C64" s="4"/>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65" s="4"/>
+      <c r="B65" s="4"/>
+      <c r="C65" s="4"/>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66" s="4"/>
+      <c r="B66" s="4"/>
+      <c r="C66" s="4"/>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67" s="4"/>
+      <c r="B67" s="4"/>
+      <c r="C67" s="4"/>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68" s="4"/>
+      <c r="B68" s="4"/>
+      <c r="C68" s="4"/>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A69" s="4"/>
+      <c r="B69" s="4"/>
+      <c r="C69" s="4"/>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A70" s="4"/>
+      <c r="B70" s="4"/>
+      <c r="C70" s="4"/>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A71" s="4"/>
+      <c r="B71" s="4"/>
+      <c r="C71" s="4"/>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A72" s="4"/>
+      <c r="B72" s="4"/>
+      <c r="C72" s="4"/>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A73" s="4"/>
+      <c r="B73" s="4"/>
+      <c r="C73" s="4"/>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A74" s="4"/>
+      <c r="B74" s="4"/>
+      <c r="C74" s="4"/>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A75" s="4"/>
+      <c r="B75" s="4"/>
+      <c r="C75" s="4"/>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A76" s="4"/>
+      <c r="B76" s="4"/>
+      <c r="C76" s="4"/>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A77" s="4"/>
+      <c r="B77" s="4"/>
+      <c r="C77" s="4"/>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A78" s="4"/>
+      <c r="B78" s="4"/>
+      <c r="C78" s="4"/>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A79" s="4"/>
+      <c r="B79" s="4"/>
+      <c r="C79" s="4"/>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A80" s="4"/>
+      <c r="B80" s="4"/>
+      <c r="C80" s="4"/>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A81" s="4"/>
+      <c r="B81" s="4"/>
+      <c r="C81" s="4"/>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A82" s="4"/>
+      <c r="B82" s="4"/>
+      <c r="C82" s="4"/>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A83" s="4"/>
+      <c r="B83" s="4"/>
+      <c r="C83" s="4"/>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A84" s="4"/>
+      <c r="B84" s="4"/>
+      <c r="C84" s="4"/>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A85" s="4"/>
+      <c r="B85" s="4"/>
+      <c r="C85" s="4"/>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A86" s="4"/>
+      <c r="B86" s="4"/>
+      <c r="C86" s="4"/>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A87" s="4"/>
+      <c r="B87" s="4"/>
+      <c r="C87" s="4"/>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A88" s="4"/>
+      <c r="B88" s="4"/>
+      <c r="C88" s="4"/>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A89" s="4"/>
+      <c r="B89" s="4"/>
+      <c r="C89" s="4"/>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A90" s="4"/>
+      <c r="B90" s="4"/>
+      <c r="C90" s="4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="D5:D7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="38.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="5" spans="4:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="D5" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="4:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="D7" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>